<commit_message>
docs: 项目计划去除 Terraform，改为 Azure CLI / Bicep 部署脚本
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report/项目执行计划.xlsx
+++ b/report/项目执行计划.xlsx
@@ -860,12 +860,12 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>① 需求分析：BRD、用户故事、验收标准、业务流程图 ② 技术架构：Azure 组件设计、Databricks 湖仓、UC 权限体系 ③ 代码评审与技术决策 ④ IaC（Terraform）⑤ 与业务方/源方/网络团队的沟通协调</t>
+          <t>① 需求分析：BRD、用户故事、验收标准、业务流程图 ② 技术架构：Azure 组件设计、Databricks 湖仓、UC 权限体系 ③ 代码评审与技术决策 ④ Azure 基础设施搭建（Azure CLI / Bicep）⑤ 与业务方/源方/网络团队的沟通协调</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>需求分析 / Databricks / Terraform / Azure 网络 / 架构设计</t>
+          <t>需求分析 / Databricks / Azure CLI / Bicep / Azure 网络 / 架构设计</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>BRD（业务需求文档）、用户故事地图、验收标准、Terraform 模块、UC 权限矩阵、架构决策记录（ADR）、部署手册</t>
+          <t>BRD（业务需求文档）、用户故事地图、验收标准、部署脚本（Azure CLI / Bicep）、UC 权限矩阵、架构决策记录（ADR）、部署手册</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>① A：BRD 初稿 + 用户故事地图 + 验收标准 + 首系统确认 ② A：Terraform 基线（VNet/AKS/ADLS/SQL DB/Key Vault/Databricks）③ B：Databricks 工作区 + UC 初始化 + 源库 PoC ④ C：项目骨架 + CI/CD 流水线 + Docker 本地开发环境 ⑤ D：测试计划 + 架构图初稿（系统上下文图 + 容器图）</t>
+          <t>① A：BRD 初稿 + 用户故事地图 + 验收标准 + 首系统确认 ② A：Azure 环境搭建（CLI/Bicep：VNet/AKS/ADLS/SQL DB/Key Vault/Databricks）③ B：Databricks 工作区 + UC 初始化 + 源库 PoC ④ C：项目骨架 + CI/CD 流水线 + Docker 本地开发环境 ⑤ D：测试计划 + 架构图初稿（系统上下文图 + 容器图）</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>① A：生产 Terraform apply + 安全评审材料 ② B：首系统全量迁移 + 生产 Jobs 部署 ③ C：生产 AKS 部署 + SSO + 监控接入 ④ D：文档冲刺（用户手册终版 + 运维手册终版 + 架构图终版 + 详细设计终版 + 接口文档终版 + 审批材料包）+ UAT 执行</t>
+          <t>① A：生产环境部署（CLI/Bicep）+ 安全评审材料 ② B：首系统全量迁移 + 生产 Jobs 部署 ③ C：生产 AKS 部署 + SSO + 监控接入 ④ D：文档冲刺（用户手册终版 + 运维手册终版 + 架构图终版 + 详细设计终版 + 接口文档终版 + 审批材料包）+ UAT 执行</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="F7" s="29" t="inlineStr">
         <is>
-          <t>ACR 先建好（A 的 Terraform）</t>
+          <t>ACR 先建好（A 的 CLI 脚本）</t>
         </is>
       </c>
       <c r="G7" s="30" t="inlineStr"/>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>① BRD 评审会（业务方确认）→ 定稿 ② 用户故事地图 + Sprint 1~6 验收标准 ③ Terraform 完整基线：VNet/AKS/ADLS/SQL DB/Key Vault/AppGateway+WAF/PE/NCC ④ IaC 部署到 Dev 环境 ⑤ UC 权限矩阵</t>
+          <t>① BRD 评审会（业务方确认）→ 定稿 ② 用户故事地图 + Sprint 1~6 验收标准 ③ Azure CLI 完整脚本：VNet/AKS/ADLS/SQL DB/Key Vault/AppGateway+WAF/PE/NCC ④ 部署到 Dev 环境 ⑤ UC 权限矩阵</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="C37" s="27" t="inlineStr">
         <is>
-          <t>① 生产 Terraform Review + apply ② 安全评审材料（等保/个保法对照表）③ 生产域名/证书/网络确认 ④ 全量迁移方案</t>
+          <t>① 生产环境部署（CLI/Bicep 脚本执行）② 安全评审材料（等保/个保法对照表）③ 生产域名/证书/网络确认 ④ 全量迁移方案</t>
         </is>
       </c>
       <c r="D37" s="28" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Terraform/部署全部阻塞</t>
+          <t>Azure 环境搭建/部署全部阻塞</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs: CI/CD 工具改为 Azure DevOps Pipelines
- GitHub Actions 全部替换为 Azure DevOps Pipelines（4 处）
- W1 CI 骨架：Azure Pipelines + 平台 ACR + DevOps Repo 连接
- W2 CD 流水线：Azure DevOps Environments + Helm 部署平台 AKS
  （服务连接走托管标识）
- Sheet1 D 角色职责与技能同步：YAML Pipeline / Environments 多环境审批

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report/项目执行计划.xlsx
+++ b/report/项目执行计划.xlsx
@@ -1920,6 +1920,7 @@
         <v>3300</v>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2109,12 +2110,12 @@
       </c>
       <c r="C8" s="43" t="inlineStr">
         <is>
-          <t>① .NET 10 后端：元数据服务 + 查询代理（SQL 拼装与白名单校验）+ 附件服务（SAS 签发）+ 调度服务 ② React 前端：配置化查询平台（JSON Schema 动态渲染）③ CI/CD：GitHub Actions → ACR → Helm 部署到平台提供的 AKS 命名空间（多环境 values）④ 代码安全四道门禁：SAST（CodeQL/Semgrep）、依赖漏洞扫描（Dependabot/audit）、密钥泄漏扫描（gitleaks）、镜像 CVE 扫描（Trivy）—— CI 强制卡点 + 高中危清零 ⑤ SSO 集成（Entra ID OIDC + JWT 角色 Claims）</t>
+          <t>① .NET 10 后端：元数据服务 + 查询代理（SQL 拼装与白名单校验）+ 附件服务（SAS 签发）+ 调度服务 ② React 前端：配置化查询平台（JSON Schema 动态渲染）③ CI/CD：Azure DevOps Pipelines → ACR → Helm 部署到平台提供的 AKS 命名空间（多环境 values）④ 代码安全四道门禁：SAST（CodeQL/Semgrep）、依赖漏洞扫描（Dependabot/audit）、密钥泄漏扫描（gitleaks）、镜像 CVE 扫描（Trivy）—— CI 强制卡点 + 高中危清零 ⑤ SSO 集成（Entra ID OIDC + JWT 角色 Claims）</t>
         </is>
       </c>
       <c r="D8" s="33" t="inlineStr">
         <is>
-          <t>.NET 10 / React / Docker / Helm / GitHub Actions / AKS / OIDC</t>
+          <t>.NET 10 / React / Docker / Helm / Azure DevOps Pipelines / AKS / OIDC</t>
         </is>
       </c>
       <c r="E8" s="44">
@@ -2203,6 +2204,7 @@
       <c r="H10" s="53" t="n"/>
       <c r="I10" s="53" t="n"/>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr"/>
     </row>
@@ -3332,7 +3334,7 @@
       <c r="C17" s="88" t="n"/>
       <c r="D17" s="78" t="inlineStr">
         <is>
-          <t>• CI 骨架：GitHub Actions build + 单测 + 推镜像（平台 ACR）</t>
+          <t>• CI 骨架：Azure DevOps Pipelines build + 单测 + 推镜像（平台 ACR）</t>
         </is>
       </c>
       <c r="E17" s="81" t="n"/>
@@ -3604,7 +3606,7 @@
       </c>
       <c r="D29" s="78" t="inlineStr">
         <is>
-          <t>• CD 流水线：Helm 部署到平台 AKS 的 Dev 命名空间</t>
+          <t>• CD 流水线：Azure DevOps Environments（Dev）+ Helm 部署到平台 AKS 命名空间（服务连接走托管标识）</t>
         </is>
       </c>
       <c r="E29" s="79" t="inlineStr">

</xml_diff>

<commit_message>
fix: 周计划 W12 的 Release 标记修正为 R2
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report/项目执行计划.xlsx
+++ b/report/项目执行计划.xlsx
@@ -7313,7 +7313,7 @@
     <row r="163" ht="22" customHeight="1">
       <c r="A163" s="118" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B163" s="95" t="inlineStr">
@@ -7379,7 +7379,7 @@
     <row r="166" ht="22" customHeight="1">
       <c r="A166" s="118" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B166" s="95" t="inlineStr">
@@ -7430,7 +7430,7 @@
     <row r="168" ht="22" customHeight="1">
       <c r="A168" s="118" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B168" s="95" t="inlineStr">
@@ -7481,7 +7481,7 @@
     <row r="170" ht="22" customHeight="1">
       <c r="A170" s="118" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B170" s="95" t="inlineStr">
@@ -7532,7 +7532,7 @@
     <row r="172" ht="22" customHeight="1">
       <c r="A172" s="118" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B172" s="95" t="inlineStr">

</xml_diff>